<commit_message>
Re-verify base contacts and add Miles Import to client list
Contacts of the 36 base companies re-checked against official pages
(25.10.2026): new emails found for Cobana and Compagnie Fruitiere, personal
address of Werder Frucht replaced by the company one, three Dole entries
flagged as not confirmed. Miles Import added as a separate client.

Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WwBoJzofjtAGn8SmQtUkmd
</commit_message>
<xml_diff>
--- a/Бананы_клиенты/Клиенты_подписка_на_цены_бананов.xlsx
+++ b/Бананы_клиенты/Клиенты_подписка_на_цены_бананов.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Как читать" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Независимые'!$A$1:$L$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Независимые'!$A$1:$L$35</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Группы (второй этап)'!$A$1:$M$26</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -128,11 +128,11 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -508,7 +508,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L34"/>
+  <dimension ref="A1:L35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -631,15 +631,19 @@
       </c>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t>https://citronex.pl/pl/</t>
+          <t>https://citronex.pl/pl/kontakt</t>
         </is>
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
-          <t>по документу (раздел 4), в этой сессии не перепроверялось</t>
-        </is>
-      </c>
-      <c r="L2" s="3" t="inlineStr"/>
+          <t>перепроверено 25.10.2026: совпадает с официальной страницей (по выдаче поиска)</t>
+        </is>
+      </c>
+      <c r="L2" s="3" t="inlineStr">
+        <is>
+          <t>На странице контактов телефон записан как +48 75 77 21 940 (тот же номер), второй номер +48 75 77 21 946. У дочерних структур группы свои телефоны, это головной офис.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -748,10 +752,14 @@
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>по документу (раздел 4), в этой сессии не перепроверялось</t>
-        </is>
-      </c>
-      <c r="L4" s="3" t="inlineStr"/>
+          <t>перепроверено 25.10.2026: совпадает с официальной страницей (по выдаче поиска)</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>Офис Dolzago. Телефоны рыночных точек: Милан +39 02 59900797, Верона +39 045 8621444.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -780,26 +788,34 @@
           <t>A</t>
         </is>
       </c>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>нет (по документу: через LinkedIn)</t>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>investor.relations@orserogroup.it (только для инвесторов, коммерческого адреса нет)</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I5" s="3" t="inlineStr"/>
-      <c r="J5" s="3" t="inlineStr"/>
+          <t>+39 0182 560400</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>https://www.orserogroup.it</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>https://emarketstorage.it/sites/default/files/comunicati/2022-03/20220318_109835.pdf</t>
+        </is>
+      </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>по документу; в этой сессии не перепроверялось</t>
+          <t>найдено при перепроверке 25.10.2026 (один источник)</t>
         </is>
       </c>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>Своя логистика и аналитика, возможна вторая волна продаж.</t>
+          <t>Найдено при перепроверке в пресс-релизе Orsero за 2022 г. (страница не открывалась): телефон и адрес для связи с инвесторами, актуальность неизвестна. Для продаж нужен личный выход через LinkedIn. Своя логистика и аналитика, возможна вторая волна продаж.</t>
         </is>
       </c>
     </row>
@@ -847,15 +863,19 @@
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>https://www.agrofair.nl</t>
+          <t>https://www.agrofair.nl/contact-us/</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>по документу (раздел 4), в этой сессии не перепроверялось</t>
-        </is>
-      </c>
-      <c r="L6" s="3" t="inlineStr"/>
+          <t>перепроверено 25.10.2026: совпадает с официальной страницей (по выдаче поиска)</t>
+        </is>
+      </c>
+      <c r="L6" s="3" t="inlineStr">
+        <is>
+          <t>Адрес: Koopliedenweg 10, 2991 LN Barendrecht.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -901,17 +921,17 @@
       </c>
       <c r="J7" s="5" t="inlineStr">
         <is>
-          <t>https://port-international.com/impressum/</t>
+          <t>https://port-international.com/en/legal-notice/</t>
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>по документу (раздел 4), в этой сессии не перепроверялось</t>
+          <t>перепроверено 25.10.2026: совпадает с официальной страницей (по выдаче поиска)</t>
         </is>
       </c>
       <c r="L7" s="3" t="inlineStr">
         <is>
-          <t>Германия: холодный рекламный email запрещён (UWG §7), первое касание через LinkedIn или звонок.</t>
+          <t>Страница в поисковом индексе примерно двухлетней давности. Адрес: Lippeltstr. 1, 20097 Hamburg. Германия: холодный рекламный email запрещён (UWG §7), первое касание через LinkedIn или звонок.</t>
         </is>
       </c>
     </row>
@@ -942,9 +962,9 @@
           <t>A</t>
         </is>
       </c>
-      <c r="G8" s="6" t="inlineStr">
-        <is>
-          <t>нет (сайт блокирует автодоступ)</t>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>info@cobana.com</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
@@ -952,20 +972,24 @@
           <t>+49 40 30305-0</t>
         </is>
       </c>
-      <c r="I8" s="3" t="inlineStr"/>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>https://www.cobana.com</t>
+        </is>
+      </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
-          <t>https://www.cio.de/article/3701022/cobana-gmbh-und-co-kg-it-fakten-und-it-strategie.html</t>
+          <t>https://www.cobana.com/en/contact/</t>
         </is>
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>по документу (раздел 4), в этой сессии не перепроверялось</t>
+          <t>найдено при перепроверке 25.10.2026: email и телефон совпали на нескольких страницах cobana.com</t>
         </is>
       </c>
       <c r="L8" s="3" t="inlineStr">
         <is>
-          <t>Самая ценная точка в Германии: одна сделка с союзом даёт выход на сеть его оптовиков. Членство отдельных компаний проверять отдельно. Германия: холодный рекламный email запрещён (UWG §7), первое касание через LinkedIn или звонок.</t>
+          <t>В документе email не был найден (сайт блокировал автодоступ), при перепроверке адрес найден. Адрес: Neue Burg 2, 20457 Hamburg. Самая ценная точка в Германии: одна сделка с союзом даёт выход на сеть его оптовиков. Германия: холодный рекламный email запрещён (UWG §7), первое касание через LinkedIn или звонок.</t>
         </is>
       </c>
     </row>
@@ -998,7 +1022,7 @@
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>info@shp-group.co.uk</t>
+          <t>info@shp-group.co.uk (не подтверждён: на сайте скрыт)</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
@@ -1013,15 +1037,19 @@
       </c>
       <c r="J9" s="5" t="inlineStr">
         <is>
-          <t>https://www.shp-group.co.uk</t>
+          <t>https://www.shp-group.co.uk/contact/</t>
         </is>
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>по документу (раздел 4), в этой сессии не перепроверялось</t>
-        </is>
-      </c>
-      <c r="L9" s="3" t="inlineStr"/>
+          <t>перепроверено 25.10.2026: часть данных совпала, см. примечание</t>
+        </is>
+      </c>
+      <c r="L9" s="3" t="inlineStr">
+        <is>
+          <t>Телефон подтверждён. В отчёте ESG 2022/23 группы указан другой адрес info@shprattgroup.com, проверить на сайте перед рассылкой.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -1335,7 +1363,7 @@
           <t>бананы ~30% выручки, сеть дозревания (74% у Fyffes)</t>
         </is>
       </c>
-      <c r="F15" s="7" t="inlineStr">
+      <c r="F15" s="6" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -1357,17 +1385,17 @@
       </c>
       <c r="J15" s="5" t="inlineStr">
         <is>
-          <t>https://www.vanwylick.de</t>
+          <t>https://www.vanwylick.de/en/contact/</t>
         </is>
       </c>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t>по документу (раздел 4), в этой сессии не перепроверялось</t>
+          <t>перепроверено 25.10.2026: совпадает с официальной страницей (по выдаче поиска)</t>
         </is>
       </c>
       <c r="L15" s="3" t="inlineStr">
         <is>
-          <t>Германия: холодный рекламный email запрещён (UWG §7), первое касание через LinkedIn или звонок.</t>
+          <t>Адрес: Rolandstr. 44, 40476 Düsseldorf. На сайте есть отдельные адреса для закупок, прямых продаж и торговли бананами. Германия: холодный рекламный email запрещён (UWG §7), первое касание через LinkedIn или звонок.</t>
         </is>
       </c>
     </row>
@@ -1393,35 +1421,39 @@
           <t>оптовик с дозревательной, член группы Cobana</t>
         </is>
       </c>
-      <c r="F16" s="7" t="inlineStr">
+      <c r="F16" s="6" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>s.schornberg@vsholding.de</t>
+          <t>info@werder-frucht.de</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I16" s="3" t="inlineStr"/>
+          <t>+49 33207 370-0</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>https://www.werder-frucht.de</t>
+        </is>
+      </c>
       <c r="J16" s="5" t="inlineStr">
         <is>
-          <t>https://www.uni-potsdam.de/de/wirtschaft-transfer-gesellschaft/piw/partner/werder-frucht-gmbh</t>
+          <t>https://www.werder-frucht.de/kontakt</t>
         </is>
       </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t>по документу (раздел 4), в этой сессии не перепроверялось</t>
+          <t>найдено при перепроверке 25.10.2026 на официальном сайте (в выдаче поиска только этот источник)</t>
         </is>
       </c>
       <c r="L16" s="3" t="inlineStr">
         <is>
-          <t>Личный адрес сотрудника из публичного каталога партнёров Потсдамского университета: писать адресно и аккуратно. Германия: холодный рекламный email запрещён (UWG §7), первое касание через LinkedIn или звонок.</t>
+          <t>Личный адрес сотрудника из документа заменён общим адресом компании. Для торговли и общепита: gastro@werder-frucht.de. Адрес: Am Frucht- und Frachthof 6, 14550 Groß Kreutz. Член группы Cobana (по странице Потсдамского университета). Германия: холодный рекламный email запрещён (UWG §7), первое касание через LinkedIn или звонок.</t>
         </is>
       </c>
     </row>
@@ -1447,7 +1479,7 @@
           <t>дозреватель и оптовик с 1990 г., 30 тыс. коробок в неделю (сайт), точка на рынке Бронише, прямой импорт не подтверждён</t>
         </is>
       </c>
-      <c r="F17" s="7" t="inlineStr">
+      <c r="F17" s="6" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -1505,7 +1537,7 @@
           <t>оптовик плодоовощей с дозреванием, ~20 тыс. коробок зелёных бананов в неделю, дозревание 11 тыс. коробок в неделю (сайт, страница старая), прямой импорт не подтверждён</t>
         </is>
       </c>
-      <c r="F18" s="7" t="inlineStr">
+      <c r="F18" s="6" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -1563,7 +1595,7 @@
           <t>импортёр (по сайту, прямые поставки из Южной Америки), дозреватель и оптовик, более 500 контейнеров в год (сайт)</t>
         </is>
       </c>
-      <c r="F19" s="7" t="inlineStr">
+      <c r="F19" s="6" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -1621,7 +1653,7 @@
           <t>импортёр и дозреватель, 6 камер, 10 тыс. коробок в неделю, до 20 тыс. с партнёрами, поставки в Литву, Латвию и Эстонию (сайт)</t>
         </is>
       </c>
-      <c r="F20" s="7" t="inlineStr">
+      <c r="F20" s="6" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -1679,7 +1711,7 @@
           <t>оптовик плодоовощей (группа Veikko Laine Oy, Финляндия), своя дозревалка бананов, по сайту единственная специализированная в Эстонии, объём бананов не указан</t>
         </is>
       </c>
-      <c r="F21" s="7" t="inlineStr">
+      <c r="F21" s="6" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -1737,12 +1769,12 @@
           <t>импортёр, оптовик и дозреватель, 14 камер, 10 тыс. коробок одновременно (сайт)</t>
         </is>
       </c>
-      <c r="F22" s="7" t="inlineStr">
+      <c r="F22" s="6" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G22" s="6" t="inlineStr">
+      <c r="G22" s="7" t="inlineStr">
         <is>
           <t>нет (на сайте контакты только по телефонам)</t>
         </is>
@@ -1795,7 +1827,7 @@
           <t>оптовик и импортёр плодоовощей с 1992 г.; по торговым записям Panjiva (данные из выдачи поиска) бананы - топ-товар, поставки из Южной Америки; дозревание не подтверждено</t>
         </is>
       </c>
-      <c r="F23" s="7" t="inlineStr">
+      <c r="F23" s="6" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -1853,12 +1885,12 @@
           <t>по Baltic Times связанная компания Latbana Baltic ввозила эквадорские бананы для сети Maxima Latvija (что это одно юрлицо, не подтверждено), выручка 2024 около 10,7 млн EUR (агрегатор), дозревание и объём бананов не подтверждены</t>
         </is>
       </c>
-      <c r="F24" s="7" t="inlineStr">
+      <c r="F24" s="6" t="inlineStr">
         <is>
           <t>B (предв.)</t>
         </is>
       </c>
-      <c r="G24" s="6" t="inlineStr">
+      <c r="G24" s="7" t="inlineStr">
         <is>
           <t>нет (сайт не найден)</t>
         </is>
@@ -1889,76 +1921,78 @@
       <c r="A25" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="2" t="n">
-        <v>35</v>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>нет (новая)</t>
+        </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>BAMA Gruppen</t>
+          <t>Miles Import SA</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>Норвегия, Осло</t>
+          <t>Франция, Иль-де-Франс (адрес из таможенной записи 2023: Chevilly-Larue, не подтверждён)</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>крупнейший частный дистрибьютор плодоовощей, свои дозревательные</t>
-        </is>
-      </c>
-      <c r="F25" s="8" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="G25" s="6" t="inlineStr">
-        <is>
-          <t>нет (форма на bama.no)</t>
+          <t>французский импортёр и дистрибьютор, основан в 1994 г. (цитрусовые, виноград, манго авиадоставкой), с 2020 г. развивает бренд Fyffes во Франции; с 01.01.2027 станет единственным дистрибьютором Fyffes во Франции по трёхлетнему соглашению (анонс 14.10.2026), бананы и ананасы; наличие собственной дозревалки не подтверждено</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>B (предв.)</t>
+        </is>
+      </c>
+      <c r="G25" s="7" t="inlineStr">
+        <is>
+          <t>нет (не найден)</t>
         </is>
       </c>
       <c r="H25" s="3" t="inlineStr">
         <is>
-          <t>+47 22 88 05 00</t>
-        </is>
-      </c>
-      <c r="I25" s="5" t="inlineStr">
-        <is>
-          <t>https://www.bama.no</t>
-        </is>
-      </c>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="I25" s="3" t="inlineStr"/>
       <c r="J25" s="5" t="inlineStr">
         <is>
-          <t>https://www.bama.no</t>
+          <t>https://retailtimes.co.uk/fyffes-and-miles-import-announce-strategic-partnership-in-france/</t>
         </is>
       </c>
       <c r="K25" s="3" t="inlineStr">
         <is>
-          <t>по документу (раздел 4), в этой сессии не перепроверялось</t>
-        </is>
-      </c>
-      <c r="L25" s="3" t="inlineStr"/>
+          <t>контактов не найдено при поиске 25.10.2026; существование и роль подтверждены сообщениями прессы (в выдаче поиска, страницы не открывались)</t>
+        </is>
+      </c>
+      <c r="L25" s="3" t="inlineStr">
+        <is>
+          <t>Председатель и CEO по заявлению Miles Import в пресс-релизе: Guy Lesvenan. Контакты искать через реестр Infogreffe или SIRENE и LinkedIn. Сообщали также FreshPlaza, Fruitnet, Lebensmittelpraxis.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
         <v>25</v>
       </c>
       <c r="B26" s="2" t="n">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Baltic Fresh Fruit UAB</t>
+          <t>BAMA Gruppen</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>Литва, Laistai (р-н Клайпеды), склад в Вильнюсе</t>
+          <t>Норвегия, Осло</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>импортёр плодоовощей широкого ассортимента, бананы лишь часть ассортимента, в вильнюсском складе (3,7 тыс. м²) есть система дозревания бананов (сайт), объём бананов не указан</t>
+          <t>крупнейший частный дистрибьютор плодоовощей, свои дозревательные</t>
         </is>
       </c>
       <c r="F26" s="8" t="inlineStr">
@@ -1966,34 +2000,34 @@
           <t>C</t>
         </is>
       </c>
-      <c r="G26" s="3" t="inlineStr">
-        <is>
-          <t>info@bff.lt</t>
+      <c r="G26" s="7" t="inlineStr">
+        <is>
+          <t>нет (форма на bama.no)</t>
         </is>
       </c>
       <c r="H26" s="3" t="inlineStr">
         <is>
-          <t>+370 46 215572</t>
+          <t>+47 22 88 05 00</t>
         </is>
       </c>
       <c r="I26" s="5" t="inlineStr">
         <is>
-          <t>https://bff.lt</t>
+          <t>https://www.bama.no</t>
         </is>
       </c>
       <c r="J26" s="5" t="inlineStr">
         <is>
-          <t>https://bff.lt/en/contact-us/</t>
+          <t>https://www.bama.no/kontakt-oss</t>
         </is>
       </c>
       <c r="K26" s="3" t="inlineStr">
         <is>
-          <t>подтверждено двумя независимыми поисками, 25.10.2026</t>
+          <t>перепроверено 25.10.2026: совпадает с официальной страницей (по выдаче поиска)</t>
         </is>
       </c>
       <c r="L26" s="3" t="inlineStr">
         <is>
-          <t>Закупки цитрусовых и бананов ведёт отдельный сотрудник, его личные контакты в файл не включены.</t>
+          <t>Телефон подтверждён, email на сайте не показан, только формы обращения.</t>
         </is>
       </c>
     </row>
@@ -2002,21 +2036,21 @@
         <v>26</v>
       </c>
       <c r="B27" s="2" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>A Fruits SIA</t>
+          <t>Baltic Fresh Fruit UAB</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>Латвия, Рига</t>
+          <t>Литва, Laistai (р-н Клайпеды), склад в Вильнюсе</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>оптовик фруктов с 2013 г., специализированные системы дозревания бананов (сайт), поставки сетям Латвии, Литвы и Эстонии, объём и число камер не указаны</t>
+          <t>импортёр плодоовощей широкого ассортимента, бананы лишь часть ассортимента, в вильнюсском складе (3,7 тыс. м²) есть система дозревания бананов (сайт), объём бананов не указан</t>
         </is>
       </c>
       <c r="F27" s="8" t="inlineStr">
@@ -2026,22 +2060,22 @@
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>info@afruits.lv</t>
+          <t>info@bff.lt</t>
         </is>
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>+371 675 40 098</t>
+          <t>+370 46 215572</t>
         </is>
       </c>
       <c r="I27" s="5" t="inlineStr">
         <is>
-          <t>https://afruits.lv</t>
+          <t>https://bff.lt</t>
         </is>
       </c>
       <c r="J27" s="5" t="inlineStr">
         <is>
-          <t>https://afruits.lv/en/about-us/</t>
+          <t>https://bff.lt/en/contact-us/</t>
         </is>
       </c>
       <c r="K27" s="3" t="inlineStr">
@@ -2049,28 +2083,32 @@
           <t>подтверждено двумя независимыми поисками, 25.10.2026</t>
         </is>
       </c>
-      <c r="L27" s="3" t="inlineStr"/>
+      <c r="L27" s="3" t="inlineStr">
+        <is>
+          <t>Закупки цитрусовых и бананов ведёт отдельный сотрудник, его личные контакты в файл не включены.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
         <v>27</v>
       </c>
       <c r="B28" s="2" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Fruit-Expert Poland Sp. z o.o.</t>
+          <t>A Fruits SIA</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Польша, Забже</t>
+          <t>Латвия, Рига</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>оптовик бананов и дозреватель с 1991 г., 10 камер, склад на 30 тыс. коробок (данные из профиля на job-портале); вероятно, преемник Banalux (тот же адрес в Забже, banalux.pl, biuro@banalux.pl найден одним поиском), по косвенным признакам, не подтверждено</t>
+          <t>оптовик фруктов с 2013 г., специализированные системы дозревания бананов (сайт), поставки сетям Латвии, Литвы и Эстонии, объём и число камер не указаны</t>
         </is>
       </c>
       <c r="F28" s="8" t="inlineStr">
@@ -2078,53 +2116,53 @@
           <t>C</t>
         </is>
       </c>
-      <c r="G28" s="6" t="inlineStr">
-        <is>
-          <t>нет (сайт fruit-expert.pl не открылся)</t>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>info@afruits.lv</t>
         </is>
       </c>
       <c r="H28" s="3" t="inlineStr">
         <is>
-          <t>нет</t>
-        </is>
-      </c>
-      <c r="I28" s="3" t="inlineStr"/>
+          <t>+371 675 40 098</t>
+        </is>
+      </c>
+      <c r="I28" s="5" t="inlineStr">
+        <is>
+          <t>https://afruits.lv</t>
+        </is>
+      </c>
       <c r="J28" s="5" t="inlineStr">
         <is>
-          <t>https://www.aplikuj.pl/pracodawca/347805/fruit-expert-poland-spolka-z-ograniczona-odpowiedzialnoscia</t>
+          <t>https://afruits.lv/en/about-us/</t>
         </is>
       </c>
       <c r="K28" s="3" t="inlineStr">
         <is>
-          <t>не перепроверялось</t>
-        </is>
-      </c>
-      <c r="L28" s="3" t="inlineStr">
-        <is>
-          <t>Контактов нет, источник подтверждает только существование компании.</t>
-        </is>
-      </c>
+          <t>подтверждено двумя независимыми поисками, 25.10.2026</t>
+        </is>
+      </c>
+      <c r="L28" s="3" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
         <v>28</v>
       </c>
       <c r="B29" s="2" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Elbana</t>
+          <t>Fruit-Expert Poland Sp. z o.o.</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>Польша, Краков</t>
+          <t>Польша, Забже</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>дозреватель, 7 камер давления, 8,4 тыс. коробок, более 15 лет (сайт), продаёт бананы Dole, Chiquita, Del Monte, UTC, собственный импорт не подтверждён</t>
+          <t>оптовик бананов и дозреватель с 1991 г., 10 камер, склад на 30 тыс. коробок (данные из профиля на job-портале); вероятно, преемник Banalux (тот же адрес в Забже, banalux.pl, biuro@banalux.pl найден одним поиском), по косвенным признакам, не подтверждено</t>
         </is>
       </c>
       <c r="F29" s="8" t="inlineStr">
@@ -2132,34 +2170,30 @@
           <t>C</t>
         </is>
       </c>
-      <c r="G29" s="6" t="inlineStr">
-        <is>
-          <t>нет (на найденных страницах не показан)</t>
+      <c r="G29" s="7" t="inlineStr">
+        <is>
+          <t>нет (сайт fruit-expert.pl не открылся)</t>
         </is>
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
-          <t>+48 12 659 08 69</t>
-        </is>
-      </c>
-      <c r="I29" s="5" t="inlineStr">
-        <is>
-          <t>https://www.elbana.pl</t>
-        </is>
-      </c>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="I29" s="3" t="inlineStr"/>
       <c r="J29" s="5" t="inlineStr">
         <is>
-          <t>https://www.elbana.pl/index.php?action=kontakt</t>
+          <t>https://www.aplikuj.pl/pracodawca/347805/fruit-expert-poland-spolka-z-ograniczona-odpowiedzialnoscia</t>
         </is>
       </c>
       <c r="K29" s="3" t="inlineStr">
         <is>
-          <t>найдено одним поиском, 25.10.2026</t>
+          <t>не перепроверялось</t>
         </is>
       </c>
       <c r="L29" s="3" t="inlineStr">
         <is>
-          <t>Второй телефон: +48 12 650 54 50.</t>
+          <t>Контактов нет, источник подтверждает только существование компании.</t>
         </is>
       </c>
     </row>
@@ -2168,21 +2202,21 @@
         <v>29</v>
       </c>
       <c r="B30" s="2" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>AS Bambona</t>
+          <t>Elbana</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>Эстония, Таллин</t>
+          <t>Польша, Краков</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>оптовик-импортёр плодоовощей с 1994 г., продаёт бананы коробками по 18 кг, прямой импорт и дозревание не подтверждены, бананы лишь часть ассортимента</t>
+          <t>дозреватель, 7 камер давления, 8,4 тыс. коробок, более 15 лет (сайт), продаёт бананы Dole, Chiquita, Del Monte, UTC, собственный импорт не подтверждён</t>
         </is>
       </c>
       <c r="F30" s="8" t="inlineStr">
@@ -2190,34 +2224,34 @@
           <t>C</t>
         </is>
       </c>
-      <c r="G30" s="3" t="inlineStr">
-        <is>
-          <t>tallinn@bambona.com (ящик склада)</t>
+      <c r="G30" s="7" t="inlineStr">
+        <is>
+          <t>нет (на найденных страницах не показан)</t>
         </is>
       </c>
       <c r="H30" s="3" t="inlineStr">
         <is>
-          <t>+372 605 5994</t>
+          <t>+48 12 659 08 69</t>
         </is>
       </c>
       <c r="I30" s="5" t="inlineStr">
         <is>
-          <t>https://bambona.ee</t>
+          <t>https://www.elbana.pl</t>
         </is>
       </c>
       <c r="J30" s="5" t="inlineStr">
         <is>
-          <t>https://bambona.ee/kontakt/</t>
+          <t>https://www.elbana.pl/index.php?action=kontakt</t>
         </is>
       </c>
       <c r="K30" s="3" t="inlineStr">
         <is>
-          <t>подтверждено двумя независимыми поисками, 25.10.2026</t>
+          <t>найдено одним поиском, 25.10.2026</t>
         </is>
       </c>
       <c r="L30" s="3" t="inlineStr">
         <is>
-          <t>Есть также tartu@bambona.com. Основной телефон по реестру: +372 605 5666.</t>
+          <t>Второй телефон: +48 12 650 54 50.</t>
         </is>
       </c>
     </row>
@@ -2226,21 +2260,21 @@
         <v>30</v>
       </c>
       <c r="B31" s="2" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>UAB Kauno vaisių ir daržovių prekyba</t>
+          <t>AS Bambona</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>Литва, Каунас</t>
+          <t>Эстония, Таллин</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>оптовик плодоовощей для сетей Литвы и ЕС (30 тыс. т продукции в год по всем товарам, самозаявление), бананы только в каталоге товаров, импорт и дозревание не подтверждены</t>
+          <t>оптовик-импортёр плодоовощей с 1994 г., продаёт бананы коробками по 18 кг, прямой импорт и дозревание не подтверждены, бананы лишь часть ассортимента</t>
         </is>
       </c>
       <c r="F31" s="8" t="inlineStr">
@@ -2250,51 +2284,55 @@
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>info@kvdp.lt</t>
+          <t>tallinn@bambona.com (ящик склада)</t>
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>+370 37 40 00 10</t>
+          <t>+372 605 5994</t>
         </is>
       </c>
       <c r="I31" s="5" t="inlineStr">
         <is>
-          <t>https://www.kaunovaisiai.lt</t>
+          <t>https://bambona.ee</t>
         </is>
       </c>
       <c r="J31" s="5" t="inlineStr">
         <is>
-          <t>https://www.kaunovaisiai.lt/kontaktai.html</t>
+          <t>https://bambona.ee/kontakt/</t>
         </is>
       </c>
       <c r="K31" s="3" t="inlineStr">
         <is>
-          <t>найдено одним поиском, 25.10.2026</t>
-        </is>
-      </c>
-      <c r="L31" s="3" t="inlineStr"/>
+          <t>подтверждено двумя независимыми поисками, 25.10.2026</t>
+        </is>
+      </c>
+      <c r="L31" s="3" t="inlineStr">
+        <is>
+          <t>Есть также tartu@bambona.com. Основной телефон по реестру: +372 605 5666.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
         <v>31</v>
       </c>
       <c r="B32" s="2" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>PPUH Polmex Sp. z o.o.</t>
+          <t>UAB Kauno vaisių ir daržovių prekyba</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>Польша, Новы-Сонч (точка на Бронише)</t>
+          <t>Литва, Каунас</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>импортёр плодоовощей с 1990 г., бананы в ассортименте на сайте компании, доля бананов, объём и дозревание не найдены</t>
+          <t>оптовик плодоовощей для сетей Литвы и ЕС (30 тыс. т продукции в год по всем товарам, самозаявление), бананы только в каталоге товаров, импорт и дозревание не подтверждены</t>
         </is>
       </c>
       <c r="F32" s="8" t="inlineStr">
@@ -2304,22 +2342,22 @@
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>office@polmex.pl</t>
+          <t>info@kvdp.lt</t>
         </is>
       </c>
       <c r="H32" s="3" t="inlineStr">
         <is>
-          <t>+48 18 415 67 676</t>
+          <t>+370 37 40 00 10</t>
         </is>
       </c>
       <c r="I32" s="5" t="inlineStr">
         <is>
-          <t>https://www.polmex.pl</t>
+          <t>https://www.kaunovaisiai.lt</t>
         </is>
       </c>
       <c r="J32" s="5" t="inlineStr">
         <is>
-          <t>https://www.polmex.pl/</t>
+          <t>https://www.kaunovaisiai.lt/kontaktai.html</t>
         </is>
       </c>
       <c r="K32" s="3" t="inlineStr">
@@ -2327,32 +2365,28 @@
           <t>найдено одним поиском, 25.10.2026</t>
         </is>
       </c>
-      <c r="L32" s="3" t="inlineStr">
-        <is>
-          <t>В справочнике Бронише указан ещё bronisze@polmex.pl. На английской странице другой телефон: (18) 442-88-26.</t>
-        </is>
-      </c>
+      <c r="L32" s="3" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
         <v>32</v>
       </c>
       <c r="B33" s="2" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Fructipol Sp. z o.o.</t>
+          <t>PPUH Polmex Sp. z o.o.</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>Польша, Варшава (Бронише)</t>
+          <t>Польша, Новы-Сонч (точка на Бронише)</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>по каталогу bestfoodimporters семейный импортёр и экспортёр плодоовощей, бананы в списке товаров на странице Бронише, импорт бананов и дозревание не подтверждены</t>
+          <t>импортёр плодоовощей с 1990 г., бананы в ассортименте на сайте компании, доля бананов, объём и дозревание не найдены</t>
         </is>
       </c>
       <c r="F33" s="8" t="inlineStr">
@@ -2360,30 +2394,34 @@
           <t>C</t>
         </is>
       </c>
-      <c r="G33" s="6" t="inlineStr">
-        <is>
-          <t>нет (сайт fructi.pl по каталогу, не проверен)</t>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>office@polmex.pl</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>нет</t>
-        </is>
-      </c>
-      <c r="I33" s="3" t="inlineStr"/>
+          <t>+48 18 415 67 676</t>
+        </is>
+      </c>
+      <c r="I33" s="5" t="inlineStr">
+        <is>
+          <t>https://www.polmex.pl</t>
+        </is>
+      </c>
       <c r="J33" s="5" t="inlineStr">
         <is>
-          <t>https://www.bronisze.com.pl/sprzedawca/fructipol-sp-z-oo</t>
+          <t>https://www.polmex.pl/</t>
         </is>
       </c>
       <c r="K33" s="3" t="inlineStr">
         <is>
-          <t>не перепроверялось</t>
+          <t>найдено одним поиском, 25.10.2026</t>
         </is>
       </c>
       <c r="L33" s="3" t="inlineStr">
         <is>
-          <t>Контактов нет, источник подтверждает только существование компании.</t>
+          <t>В справочнике Бронише указан ещё bronisze@polmex.pl. На английской странице другой телефон: (18) 442-88-26.</t>
         </is>
       </c>
     </row>
@@ -2392,11 +2430,11 @@
         <v>33</v>
       </c>
       <c r="B34" s="2" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Fruco Sp. z o.o.</t>
+          <t>Fructipol Sp. z o.o.</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
@@ -2406,7 +2444,7 @@
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>по справочнику Бронише многолетний импортёр цитрусовых, бананы в списке товаров, импорт бананов и дозревание не подтверждены</t>
+          <t>по каталогу bestfoodimporters семейный импортёр и экспортёр плодоовощей, бананы в списке товаров на странице Бронише, импорт бананов и дозревание не подтверждены</t>
         </is>
       </c>
       <c r="F34" s="8" t="inlineStr">
@@ -2414,35 +2452,89 @@
           <t>C</t>
         </is>
       </c>
-      <c r="G34" s="6" t="inlineStr">
-        <is>
-          <t>нет (в справочнике только бесплатная почта)</t>
+      <c r="G34" s="7" t="inlineStr">
+        <is>
+          <t>нет (сайт fructi.pl по каталогу, не проверен)</t>
         </is>
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
-          <t>+48 22 721 60 20</t>
+          <t>нет</t>
         </is>
       </c>
       <c r="I34" s="3" t="inlineStr"/>
       <c r="J34" s="5" t="inlineStr">
         <is>
+          <t>https://www.bronisze.com.pl/sprzedawca/fructipol-sp-z-oo</t>
+        </is>
+      </c>
+      <c r="K34" s="3" t="inlineStr">
+        <is>
+          <t>не перепроверялось</t>
+        </is>
+      </c>
+      <c r="L34" s="3" t="inlineStr">
+        <is>
+          <t>Контактов нет, источник подтверждает только существование компании.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>Fruco Sp. z o.o.</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>Польша, Варшава (Бронише)</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>по справочнику Бронише многолетний импортёр цитрусовых, бананы в списке товаров, импорт бананов и дозревание не подтверждены</t>
+        </is>
+      </c>
+      <c r="F35" s="8" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="G35" s="7" t="inlineStr">
+        <is>
+          <t>нет (в справочнике только бесплатная почта)</t>
+        </is>
+      </c>
+      <c r="H35" s="3" t="inlineStr">
+        <is>
+          <t>+48 22 721 60 20</t>
+        </is>
+      </c>
+      <c r="I35" s="3" t="inlineStr"/>
+      <c r="J35" s="5" t="inlineStr">
+        <is>
           <t>https://www.bronisze.com.pl/sprzedawca/fruco-sp-z-oo</t>
         </is>
       </c>
-      <c r="K34" s="3" t="inlineStr">
+      <c r="K35" s="3" t="inlineStr">
         <is>
           <t>найдено одним поиском, 25.10.2026</t>
         </is>
       </c>
-      <c r="L34" s="3" t="inlineStr">
+      <c r="L35" s="3" t="inlineStr">
         <is>
           <t>Возможна связь с Tropical Trade (одинаковый NIP в сниппетах), не проверено.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L34"/>
+  <autoFilter ref="A1:L35"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J2" r:id="rId2"/>
@@ -2450,58 +2542,63 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J3" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I4" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J4" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J6" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J7" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J8" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J9" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J10" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J11" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I12" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J12" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I13" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J13" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J14" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J15" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J16" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J17" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J18" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J19" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J20" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I21" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J21" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J22" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J23" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J24" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J25" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J26" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J27" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J28" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I29" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J29" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I30" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J30" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I31" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J31" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I32" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J32" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J33" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J34" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J5" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J6" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J7" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J8" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J9" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J10" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J11" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I12" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J12" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I13" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J13" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J14" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J15" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I16" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J16" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J17" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J18" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J19" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J20" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I21" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J21" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J22" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J23" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J24" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J25" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J26" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J27" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I28" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J28" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J29" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I30" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J30" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I31" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J31" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I32" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J32" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I33" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J33" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J34" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J35" r:id="rId63"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2648,7 +2745,7 @@
       </c>
       <c r="L2" s="3" t="inlineStr">
         <is>
-          <t>по документу: источник - страница контактов Dole plc, страница самой компании не зафиксирована; в этой сессии не перепроверялось</t>
+          <t>перепроверено 25.10.2026: совпадает со страницей контактов Dole plc (по выдаче поиска)</t>
         </is>
       </c>
       <c r="M2" s="3" t="inlineStr"/>
@@ -2703,7 +2800,7 @@
       </c>
       <c r="L3" s="3" t="inlineStr">
         <is>
-          <t>по документу: источник - страница контактов Dole plc, страница самой компании не зафиксирована; в этой сессии не перепроверялось</t>
+          <t>перепроверено 25.10.2026: совпадает со страницей контактов Dole plc (по выдаче поиска)</t>
         </is>
       </c>
       <c r="M3" s="3" t="inlineStr"/>
@@ -2758,7 +2855,7 @@
       </c>
       <c r="L4" s="3" t="inlineStr">
         <is>
-          <t>по документу: источник - страница контактов Dole plc, страница самой компании не зафиксирована; в этой сессии не перепроверялось</t>
+          <t>перепроверено 25.10.2026: совпадает со страницей контактов Dole plc (по выдаче поиска)</t>
         </is>
       </c>
       <c r="M4" s="3" t="inlineStr"/>
@@ -2790,7 +2887,7 @@
           <t>коммерческий офис</t>
         </is>
       </c>
-      <c r="G5" s="7" t="inlineStr">
+      <c r="G5" s="6" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -2813,7 +2910,7 @@
       </c>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>по документу: источник - страница контактов Dole plc, страница самой компании не зафиксирована; в этой сессии не перепроверялось</t>
+          <t>перепроверено 25.10.2026: совпадает со страницей контактов Dole plc (по выдаче поиска)</t>
         </is>
       </c>
       <c r="M5" s="3" t="inlineStr"/>
@@ -2863,15 +2960,19 @@
       <c r="J6" s="3" t="inlineStr"/>
       <c r="K6" s="5" t="inlineStr">
         <is>
-          <t>https://www.doleplc.com/contact</t>
+          <t>https://eurobanan.com/contacto/</t>
         </is>
       </c>
       <c r="L6" s="3" t="inlineStr">
         <is>
-          <t>по документу: источник - страница контактов Dole plc, страница самой компании не зафиксирована; в этой сессии не перепроверялось</t>
-        </is>
-      </c>
-      <c r="M6" s="3" t="inlineStr"/>
+          <t>перепроверено 25.10.2026: совпадает с официальной страницей (по выдаче поиска)</t>
+        </is>
+      </c>
+      <c r="M6" s="3" t="inlineStr">
+        <is>
+          <t>У Мадрида несколько номеров: +34 91 779 66 00 (страница контактов), 917 796 600 и +34 91 779 66 72 (правовая страница).</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -2918,12 +3019,12 @@
       <c r="J7" s="3" t="inlineStr"/>
       <c r="K7" s="5" t="inlineStr">
         <is>
-          <t>https://www.doleplc.com/contact</t>
+          <t>https://eurobanan.com/contacto/</t>
         </is>
       </c>
       <c r="L7" s="3" t="inlineStr">
         <is>
-          <t>по документу: источник - страница контактов Dole plc, страница самой компании не зафиксирована; в этой сессии не перепроверялось</t>
+          <t>перепроверено 25.10.2026: совпадает с официальной страницей (по выдаче поиска)</t>
         </is>
       </c>
       <c r="M7" s="3" t="inlineStr"/>
@@ -2973,12 +3074,12 @@
       <c r="J8" s="3" t="inlineStr"/>
       <c r="K8" s="5" t="inlineStr">
         <is>
-          <t>https://www.doleplc.com/contact</t>
+          <t>https://eurobanan.com/contacto/</t>
         </is>
       </c>
       <c r="L8" s="3" t="inlineStr">
         <is>
-          <t>по документу: источник - страница контактов Dole plc, страница самой компании не зафиксирована; в этой сессии не перепроверялось</t>
+          <t>перепроверено 25.10.2026: совпадает с официальной страницей (по выдаче поиска)</t>
         </is>
       </c>
       <c r="M8" s="3" t="inlineStr"/>
@@ -3028,12 +3129,12 @@
       <c r="J9" s="3" t="inlineStr"/>
       <c r="K9" s="5" t="inlineStr">
         <is>
-          <t>https://www.doleplc.com/contact</t>
+          <t>https://eurobanan.com/contacto/</t>
         </is>
       </c>
       <c r="L9" s="3" t="inlineStr">
         <is>
-          <t>по документу: источник - страница контактов Dole plc, страница самой компании не зафиксирована; в этой сессии не перепроверялось</t>
+          <t>перепроверено 25.10.2026: совпадает с официальной страницей (по выдаче поиска)</t>
         </is>
       </c>
       <c r="M9" s="3" t="inlineStr"/>
@@ -3083,15 +3184,19 @@
       <c r="J10" s="3" t="inlineStr"/>
       <c r="K10" s="5" t="inlineStr">
         <is>
-          <t>https://www.doleplc.com/contact</t>
+          <t>https://eurobanan.com/contacto/</t>
         </is>
       </c>
       <c r="L10" s="3" t="inlineStr">
         <is>
-          <t>по документу: источник - страница контактов Dole plc, страница самой компании не зафиксирована; в этой сессии не перепроверялось</t>
-        </is>
-      </c>
-      <c r="M10" s="3" t="inlineStr"/>
+          <t>перепроверено 25.10.2026: совпадает с официальной страницей (по выдаче поиска)</t>
+        </is>
+      </c>
+      <c r="M10" s="3" t="inlineStr">
+        <is>
+          <t>На сайте два адреса в районе Виго (рынок Mercado Vigo и Centro Galicia в Порриньо) с одним email.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -3143,7 +3248,7 @@
       </c>
       <c r="L11" s="3" t="inlineStr">
         <is>
-          <t>по документу: источник - страница контактов Dole plc, страница самой компании не зафиксирована; в этой сессии не перепроверялось</t>
+          <t>email подтверждён на странице Dole plc 25.10.2026, телефон отдельно не подтверждён</t>
         </is>
       </c>
       <c r="M11" s="3" t="inlineStr"/>
@@ -3198,7 +3303,7 @@
       </c>
       <c r="L12" s="3" t="inlineStr">
         <is>
-          <t>по документу: источник - страница контактов Dole plc, страница самой компании не зафиксирована; в этой сессии не перепроверялось</t>
+          <t>email подтверждён на странице Dole plc 25.10.2026, телефон отдельно не подтверждён</t>
         </is>
       </c>
       <c r="M12" s="3" t="inlineStr"/>
@@ -3252,17 +3357,17 @@
       </c>
       <c r="K13" s="5" t="inlineStr">
         <is>
-          <t>https://www.doleplc.com/contact</t>
+          <t>https://www.anacogreeve.nl/contact/</t>
         </is>
       </c>
       <c r="L13" s="3" t="inlineStr">
         <is>
-          <t>по документу; присутствие в списке контактов Dole plc подтверждено поиском 25.10.2026, прямого подтверждения владения Dole не найдено</t>
+          <t>перепроверено 25.10.2026: совпадает с официальной страницей (по выдаче поиска)</t>
         </is>
       </c>
       <c r="M13" s="3" t="inlineStr">
         <is>
-          <t>Принадлежность к группе Dole выведена из страницы контактов Dole plc, прямое подтверждение владения не найдено.</t>
+          <t>Принадлежность к группе Dole выведена из страницы контактов Dole plc, прямое подтверждение владения не найдено. Актуальный телефон +31 174 638 666 (на старой странице другие номера). Личные адреса специалистов на сайте есть, в файл не включены.</t>
         </is>
       </c>
     </row>
@@ -3293,12 +3398,12 @@
           <t>европейский офис Dole</t>
         </is>
       </c>
-      <c r="G14" s="7" t="inlineStr">
+      <c r="G14" s="6" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="H14" s="6" t="inlineStr">
+      <c r="H14" s="7" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
@@ -3316,10 +3421,14 @@
       </c>
       <c r="L14" s="3" t="inlineStr">
         <is>
-          <t>по документу: источник - страница контактов Dole plc, страница самой компании не зафиксирована; в этой сессии не перепроверялось</t>
-        </is>
-      </c>
-      <c r="M14" s="3" t="inlineStr"/>
+          <t>перепроверено 25.10.2026: совпадает со страницей контактов Dole plc (по выдаче поиска)</t>
+        </is>
+      </c>
+      <c r="M14" s="3" t="inlineStr">
+        <is>
+          <t>Офис в Блейсвейке, email на странице не указан.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -3348,7 +3457,7 @@
           <t>штаб Dole в Германии</t>
         </is>
       </c>
-      <c r="G15" s="7" t="inlineStr">
+      <c r="G15" s="6" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -3371,7 +3480,7 @@
       </c>
       <c r="L15" s="3" t="inlineStr">
         <is>
-          <t>по документу: источник - страница контактов Dole plc, страница самой компании не зафиксирована; в этой сессии не перепроверялось</t>
+          <t>перепроверено 25.10.2026: совпадает со страницей контактов Dole plc (по выдаче поиска)</t>
         </is>
       </c>
       <c r="M15" s="3" t="inlineStr">
@@ -3407,7 +3516,7 @@
           <t>импорт и дистрибуция</t>
         </is>
       </c>
-      <c r="G16" s="7" t="inlineStr">
+      <c r="G16" s="6" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -3430,10 +3539,14 @@
       </c>
       <c r="L16" s="3" t="inlineStr">
         <is>
-          <t>по документу: источник - страница контактов Dole plc, страница самой компании не зафиксирована; в этой сессии не перепроверялось</t>
-        </is>
-      </c>
-      <c r="M16" s="3" t="inlineStr"/>
+          <t>не подтвердилось при перепроверке 25.10.2026, см. примечание</t>
+        </is>
+      </c>
+      <c r="M16" s="3" t="inlineStr">
+        <is>
+          <t>Адрес mail@totalproduce.fr и офис в Кавайоне не найдены ни на странице Dole plc, ни в других источниках. Total Produce Indigo стала Dole France с 01.01.2023 (по Réussir), головной офис Dole France: 511 Route de la Seds, 13127 Vitrolles. Возможный дубль строки 29.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -3462,7 +3575,7 @@
           <t>импорт и дистрибуция</t>
         </is>
       </c>
-      <c r="G17" s="7" t="inlineStr">
+      <c r="G17" s="6" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -3485,10 +3598,14 @@
       </c>
       <c r="L17" s="3" t="inlineStr">
         <is>
-          <t>по документу: источник - страница контактов Dole plc, страница самой компании не зафиксирована; в этой сессии не перепроверялось</t>
-        </is>
-      </c>
-      <c r="M17" s="3" t="inlineStr"/>
+          <t>не подтвердилось при перепроверке 25.10.2026, см. примечание</t>
+        </is>
+      </c>
+      <c r="M17" s="3" t="inlineStr">
+        <is>
+          <t>sales@indigo-fruit.com не подтвердился. Indigo Fruit входит в Dole France (с 01.01.2023), головной офис в Витроле. Возможный дубль строки 28.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -3517,7 +3634,7 @@
           <t>банановая компания в группе Dole</t>
         </is>
       </c>
-      <c r="G18" s="7" t="inlineStr">
+      <c r="G18" s="6" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -3540,10 +3657,14 @@
       </c>
       <c r="L18" s="3" t="inlineStr">
         <is>
-          <t>по документу: источник - страница контактов Dole plc, страница самой компании не зафиксирована; в этой сессии не перепроверялось</t>
-        </is>
-      </c>
-      <c r="M18" s="3" t="inlineStr"/>
+          <t>не подтвердилось при перепроверке 25.10.2026, см. примечание</t>
+        </is>
+      </c>
+      <c r="M18" s="3" t="inlineStr">
+        <is>
+          <t>AB Banan-Kompaniet не найдена ни на странице Dole plc, ни в поиске. Домен saba.se, по сообщению SFVBJ (из выдачи поиска, страница не открывалась), связан с Saba Fresh Cuts, которую Dole продала группе Bama, email мог устареть. Не использовать без проверки.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -3595,7 +3716,7 @@
       </c>
       <c r="L19" s="3" t="inlineStr">
         <is>
-          <t>по документу: источник - страница контактов Dole plc, страница самой компании не зафиксирована; в этой сессии не перепроверялось</t>
+          <t>перепроверено 25.10.2026: совпадает со страницей контактов Dole plc (по выдаче поиска)</t>
         </is>
       </c>
       <c r="M19" s="3" t="inlineStr"/>
@@ -3650,7 +3771,7 @@
       </c>
       <c r="L20" s="3" t="inlineStr">
         <is>
-          <t>по документу: источник - страница контактов Dole plc, страница самой компании не зафиксирована; в этой сессии не перепроверялось</t>
+          <t>перепроверено 25.10.2026: совпадает со страницей контактов Dole plc (по выдаче поиска)</t>
         </is>
       </c>
       <c r="M20" s="3" t="inlineStr"/>
@@ -3687,7 +3808,7 @@
           <t>C</t>
         </is>
       </c>
-      <c r="H21" s="6" t="inlineStr">
+      <c r="H21" s="7" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
@@ -3705,10 +3826,14 @@
       </c>
       <c r="L21" s="3" t="inlineStr">
         <is>
-          <t>по документу: источник - страница контактов Dole plc, страница самой компании не зафиксирована; в этой сессии не перепроверялось</t>
-        </is>
-      </c>
-      <c r="M21" s="3" t="inlineStr"/>
+          <t>перепроверено 25.10.2026: совпадает со страницей контактов Dole plc (по выдаче поиска)</t>
+        </is>
+      </c>
+      <c r="M21" s="3" t="inlineStr">
+        <is>
+          <t>На странице два датских адреса: Hasselager +45 86 28 82 22 и Кёге +45 36 15 63 22.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -3737,12 +3862,12 @@
           <t>европейский импорт Chiquita</t>
         </is>
       </c>
-      <c r="G22" s="7" t="inlineStr">
+      <c r="G22" s="6" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="H22" s="6" t="inlineStr">
+      <c r="H22" s="7" t="inlineStr">
         <is>
           <t>нет (по документу: через LinkedIn)</t>
         </is>
@@ -3760,7 +3885,7 @@
       </c>
       <c r="L22" s="3" t="inlineStr">
         <is>
-          <t>по документу; в этой сессии не перепроверялось</t>
+          <t>контактов нет, перепроверять нечего</t>
         </is>
       </c>
       <c r="M22" s="3" t="inlineStr"/>
@@ -3792,19 +3917,19 @@
           <t>называет себя крупнейшим дозревателем бананов в Европе</t>
         </is>
       </c>
-      <c r="G23" s="7" t="inlineStr">
+      <c r="G23" s="6" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="H23" s="6" t="inlineStr">
+      <c r="H23" s="7" t="inlineStr">
         <is>
           <t>нет (скрыт на сайте, форма greenyard.group)</t>
         </is>
       </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>+32 15 32 47 00 (Greenyard Fresh Belgium)</t>
         </is>
       </c>
       <c r="J23" s="5" t="inlineStr">
@@ -3814,15 +3939,19 @@
       </c>
       <c r="K23" s="5" t="inlineStr">
         <is>
-          <t>https://www.greenyard.group/divisions/fresh/local-pages/fresh-hq</t>
+          <t>https://www.greenyard.group/nl/divisions/fresh/local-pages/fresh-belgium</t>
         </is>
       </c>
       <c r="L23" s="3" t="inlineStr">
         <is>
-          <t>по документу (раздел 4), в этой сессии не перепроверялось</t>
-        </is>
-      </c>
-      <c r="M23" s="3" t="inlineStr"/>
+          <t>найдено при перепроверке 25.10.2026 (один источник)</t>
+        </is>
+      </c>
+      <c r="M23" s="3" t="inlineStr">
+        <is>
+          <t>Email на сайте скрыт, есть только форма. Головной офис: Strijbroek 10, Sint-Katelijne-Waver, телефон корпоративного офиса +32 15 32 42 00. Адрес info.direct@greenyardfresh.be относится к другому подразделению (Fresh Direct Belgium).</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -3851,14 +3980,14 @@
           <t>~775 тыс. т бананов в год, 22 дозревательных центра в 8 странах</t>
         </is>
       </c>
-      <c r="G24" s="7" t="inlineStr">
+      <c r="G24" s="6" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="H24" s="6" t="inlineStr">
-        <is>
-          <t>нет (не подтверждён)</t>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>fruitiere@fruitiere.fr</t>
         </is>
       </c>
       <c r="I24" s="3" t="inlineStr">
@@ -3873,15 +4002,19 @@
       </c>
       <c r="K24" s="5" t="inlineStr">
         <is>
-          <t>https://compagniefruitiere.fr/wp-content/uploads/2024/12/CIE-FRUITIERE-2024_DEPLIANT_WEB_UK.pdf</t>
+          <t>https://www.compagniefruitiere.fr/mentions-legales/</t>
         </is>
       </c>
       <c r="L24" s="3" t="inlineStr">
         <is>
-          <t>по документу (раздел 4), в этой сессии не перепроверялось</t>
-        </is>
-      </c>
-      <c r="M24" s="3" t="inlineStr"/>
+          <t>телефон совпал, email найден при перепроверке 25.10.2026 на странице mentions légales</t>
+        </is>
+      </c>
+      <c r="M24" s="3" t="inlineStr">
+        <is>
+          <t>Адрес: 33 boulevard Ferdinand de Lesseps, 13014 Marseille. В документе email был не подтверждён.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
@@ -3910,12 +4043,12 @@
           <t>дистрибуция бананов и тропиков</t>
         </is>
       </c>
-      <c r="G25" s="7" t="inlineStr">
+      <c r="G25" s="6" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="H25" s="6" t="inlineStr">
+      <c r="H25" s="7" t="inlineStr">
         <is>
           <t>нет (не подтверждён)</t>
         </is>
@@ -3933,7 +4066,7 @@
       </c>
       <c r="L25" s="3" t="inlineStr">
         <is>
-          <t>по документу (раздел 4), в этой сессии не перепроверялось</t>
+          <t>не перепроверялось (страница proveedores.com в поиске не вернулась)</t>
         </is>
       </c>
       <c r="M25" s="3" t="inlineStr"/>
@@ -3965,19 +4098,19 @@
           <t>крупный импортёр бананов в Европе; во Франции с 01.01.2027 единственным дистрибьютором станет Miles Import (анонс 14.10.2026, три года)</t>
         </is>
       </c>
-      <c r="G26" s="7" t="inlineStr">
+      <c r="G26" s="6" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="H26" s="6" t="inlineStr">
+      <c r="H26" s="7" t="inlineStr">
         <is>
           <t>нет (форма на fyffes.com)</t>
         </is>
       </c>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>+353 1 887 2700 (Дублин), +31 10 244 5300 (Роттердам)</t>
         </is>
       </c>
       <c r="J26" s="5" t="inlineStr">
@@ -3987,17 +4120,17 @@
       </c>
       <c r="K26" s="5" t="inlineStr">
         <is>
-          <t>https://www.fyffes.com</t>
+          <t>https://www.fyffes.com/contact-us-3/</t>
         </is>
       </c>
       <c r="L26" s="3" t="inlineStr">
         <is>
-          <t>по документу (раздел 4), в этой сессии не перепроверялось</t>
+          <t>найдено при перепроверке 25.10.2026 (один источник)</t>
         </is>
       </c>
       <c r="M26" s="3" t="inlineStr">
         <is>
-          <t>Miles Import (Франция) - отдельный клиент для будущей проверки, в базе его пока нет. Про Miles Import сообщали FreshPlaza, Fruitnet, Retail Times (в выдаче поиска, страницы не открывались).</t>
+          <t>Во Франции с 01.01.2027 единственным дистрибьютором станет Miles Import (анонс 14.10.2026, три года), он добавлен на лист «Независимые». Общего email для клиентов на странице контактов нет, только телефоны офисов, страница по данным поиска обновлялась больше полугода назад.</t>
         </is>
       </c>
     </row>
@@ -4095,7 +4228,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>33 компании: независимые импортёры, дозреватели и оптовики. Продавать в первую очередь, потому что у мультинационалов своя аналитика. Сортировка: приоритет A, B, C.</t>
+          <t>34 компании: независимые импортёры, дозреватели и оптовики. Продавать в первую очередь, потому что у мультинационалов своя аналитика. Сортировка: приоритет A, B, C.</t>
         </is>
       </c>
     </row>
@@ -4131,7 +4264,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Страница, на которой найден email или телефон. Для компаний 1-36 документ фиксирует главную страницу компании или страницу контактов группы, точная страница каждого email не записана. Для компаний 37-58 указана страница из выдачи поиска.</t>
+          <t>Страница, на которой найден email или телефон. Для компаний 1-36 при перепроверке 25.10.2026 указана страница контактов компании или группы, где данные совпали с документом (по выдаче поиска). Для компаний 37-58 указана страница из выдачи поиска. Для Orsero указан пресс-релиз 2022 г., для Miles Import - сообщение прессы о соглашении с Fyffes.</t>
         </is>
       </c>
     </row>
@@ -4143,7 +4276,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>«Подтверждено двумя независимыми поисками» - адрес и телефон дважды найдены в выдаче поиска по домену самой компании (25.10.2026). «Найдено одним поиском» - второго подтверждения нет. «По документу» - данные из раздела 4, в этой сессии не перепроверялись. Страницы целиком не открывались, потому что прокси блокирует сайты, выдача поиска пересказывается инструментом, поэтому перед рассылкой нужно один раз открыть страницу контактов в браузере.</t>
+          <t>«Подтверждено двумя независимыми поисками» - адрес и телефон дважды найдены в выдаче поиска по домену самой компании (25.10.2026). «Найдено одним поиском» - второго подтверждения нет. «Перепроверено 25.10.2026: совпадает» - контакт из раздела 4 найден в выдаче поиска на официальной странице и совпал с документом. «Найдено при перепроверке» - в документе контакта не было, при перепроверке найден один источник. «Не подтвердилось» - контакт из документа в поиске не найден, использовать только после ручной проверки. Страницы целиком не открывались, потому что прокси блокирует сайты, выдача поиска пересказывается инструментом, поэтому перед рассылкой нужно один раз открыть страницу контактов в браузере.</t>
         </is>
       </c>
     </row>
@@ -4155,7 +4288,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Личные адреса и мобильные телефоны сотрудников (кроме Werder Frucht, адрес из публичного каталога партнёров, он помечен). Рынок Бронише (Варшава) - оператор площадки, а не клиент. Не проверенные кандидаты (каталог eGospodarka, часть продавцов Бронише, список оптовиков Риги) в файл не вошли.</t>
+          <t>Личные адреса и мобильные телефоны сотрудников (личный адрес Werder Frucht из документа заменён общим адресом компании). Рынок Бронише (Варшава) - оператор площадки, а не клиент. Не проверенные кандидаты (каталог eGospodarka, часть продавцов Бронише, список оптовиков Риги) в файл не вошли.</t>
         </is>
       </c>
     </row>
@@ -4179,7 +4312,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Orsero и Simba S.p.A., вероятно, одна группа (не подтверждено). Fruit-Expert Poland, вероятно, преемник Banalux (не подтверждено). Принадлежность Anaco &amp; Greeve к Dole выведена из списка контактов Dole plc, прямого подтверждения владения нет. Сайты Royal Banane и Di Manno не открывались, в список не включены; Italfrutta Di Manno найдена в старой статье FreshPlaza (2018), актуальность неизвестна.</t>
+          <t>Итог перепроверки 25.10.2026: из 36 компаний раздела 4 контакты полностью совпали у 22, частично у 3 (SHP, Eurobanan Lisboa и Porto), новые контакты найдены у 6 (Orsero, Cobana, Werder Frucht, Greenyard, Compagnie Fruitière, Fyffes), не подтвердились у 3 (Dole France Кавайон, Dole France Витроль, Banan-Kompaniet), не перепроверялись или контактов нет у 2 (Compagnie Fruitière España, Chiquita Europe). Dole France Кавайон и Dole France (Indigo Fruit, Витроль), вероятно, одна компания: Indigo Fruit входит в Dole France с 01.01.2023. Orsero и Simba S.p.A., вероятно, одна группа (не подтверждено). Fruit-Expert Poland, вероятно, преемник Banalux (не подтверждено). Принадлежность Anaco &amp; Greeve к Dole выведена из списка контактов Dole plc, прямого подтверждения владения нет. Сайты Royal Banane и Di Manno не открывались, в список не включены; Italfrutta Di Manno найдена в старой статье FreshPlaza (2018), актуальность неизвестна.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Align client list with the updated document table
Miles Import gets number 59 as in the document, legend counts updated.

Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WwBoJzofjtAGn8SmQtUkmd
</commit_message>
<xml_diff>
--- a/Бананы_клиенты/Клиенты_подписка_на_цены_бананов.xlsx
+++ b/Бананы_клиенты/Клиенты_подписка_на_цены_бананов.xlsx
@@ -1921,10 +1921,8 @@
       <c r="A25" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>нет (новая)</t>
-        </is>
+      <c r="B25" s="2" t="n">
+        <v>59</v>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
@@ -4216,7 +4214,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Раздел 4 (36 компаний) и раздел 4а (22 компании) документа «Рынок бананов Европы: анализ и база импортёров»: https://claude.ai/artifact/61RLiR5jvtqbyENn8PMmXd. Раздел 4 собран в предыдущей сессии, раздел 4а - 25.10.2026.</t>
+          <t>Раздел 4 (36 компаний) и раздел 4а (23 компании: Польша, Прибалтика и Miles Import) документа «Рынок бананов Европы: анализ и база импортёров»: https://claude.ai/artifact/61RLiR5jvtqbyENn8PMmXd. Раздел 4 собран в предыдущей сессии, раздел 4а - 25.10.2026.</t>
         </is>
       </c>
     </row>

</xml_diff>